<commit_message>
New Request: warn when the download template is out of date
Add /api/template/version — a content hash of the BU's valid data (active
Master Descriptions + Freight Rates) and the template file bytes. The New
Request page fetches it, compares against the version this browser last
downloaded (localStorage), and shows a "template updated — please re-download"
hint + highlights the button only when they differ. Downloading the latest
clears it; users who never downloaded (or already have the latest) see nothing.

File is hashed by content, not mtime, so app redeploys don't flip the version.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/air-request-template_EA.xlsx
+++ b/public/air-request-template_EA.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEC0B98E-AB87-41C0-9A6B-1A6D4DE08370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C06D01C9-4811-452F-8960-D616630FC553}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EA" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="163">
   <si>
     <t>LOGISTICS</t>
   </si>
@@ -152,9 +152,6 @@
     <t>Los Angeles</t>
   </si>
   <si>
-    <t>United States</t>
-  </si>
-  <si>
     <t>G2</t>
   </si>
   <si>
@@ -170,9 +167,6 @@
     <t>Chicago</t>
   </si>
   <si>
-    <t>Australia</t>
-  </si>
-  <si>
     <t>G3</t>
   </si>
   <si>
@@ -188,9 +182,6 @@
     <t>Melbourne</t>
   </si>
   <si>
-    <t>Canada</t>
-  </si>
-  <si>
     <t>G4</t>
   </si>
   <si>
@@ -206,9 +197,6 @@
     <t>Toronto</t>
   </si>
   <si>
-    <t>United Kingdom</t>
-  </si>
-  <si>
     <t>BOXER</t>
   </si>
   <si>
@@ -218,9 +206,6 @@
     <t>Vancouver</t>
   </si>
   <si>
-    <t>Netherlands</t>
-  </si>
-  <si>
     <t>T-SHIRT</t>
   </si>
   <si>
@@ -236,27 +221,18 @@
     <t>Amsterdam</t>
   </si>
   <si>
-    <t>Japan</t>
-  </si>
-  <si>
     <t>CLAIM</t>
   </si>
   <si>
     <t>PULLOVER</t>
   </si>
   <si>
-    <t>Mexico</t>
-  </si>
-  <si>
     <t>SHIRT</t>
   </si>
   <si>
     <t>O'hare(ORD)</t>
   </si>
   <si>
-    <t>Panama</t>
-  </si>
-  <si>
     <t>PROCUREMENT</t>
   </si>
   <si>
@@ -269,9 +245,6 @@
     <t>DURHAM</t>
   </si>
   <si>
-    <t>Belgium</t>
-  </si>
-  <si>
     <t>PRODUCTION</t>
   </si>
   <si>
@@ -281,9 +254,6 @@
     <t>LOCKBOURN</t>
   </si>
   <si>
-    <t>Germany</t>
-  </si>
-  <si>
     <t>COMMERCIAL</t>
   </si>
   <si>
@@ -390,6 +360,162 @@
   </si>
   <si>
     <t>RHONE APPAREL INC.</t>
+  </si>
+  <si>
+    <t>ALGERIA</t>
+  </si>
+  <si>
+    <t>AUSTRALIA</t>
+  </si>
+  <si>
+    <t>BELGIUM</t>
+  </si>
+  <si>
+    <t>BRAZIL</t>
+  </si>
+  <si>
+    <t>CAMBODIA</t>
+  </si>
+  <si>
+    <t>CANADA</t>
+  </si>
+  <si>
+    <t>CHILE</t>
+  </si>
+  <si>
+    <t>CHINA</t>
+  </si>
+  <si>
+    <t>COLOMBIA</t>
+  </si>
+  <si>
+    <t>COSTA RICA</t>
+  </si>
+  <si>
+    <t>DOMINICA</t>
+  </si>
+  <si>
+    <t>EL SALVADOR</t>
+  </si>
+  <si>
+    <t>FRANCE</t>
+  </si>
+  <si>
+    <t>GERMANY</t>
+  </si>
+  <si>
+    <t>HAITI</t>
+  </si>
+  <si>
+    <t>HONG KONG</t>
+  </si>
+  <si>
+    <t>INDIA</t>
+  </si>
+  <si>
+    <t>INDONESIA</t>
+  </si>
+  <si>
+    <t>IRELAND</t>
+  </si>
+  <si>
+    <t>ITALY</t>
+  </si>
+  <si>
+    <t>JAPAN</t>
+  </si>
+  <si>
+    <t>JORDAN</t>
+  </si>
+  <si>
+    <t>KOREA</t>
+  </si>
+  <si>
+    <t>LAOS</t>
+  </si>
+  <si>
+    <t>MALAYSIA</t>
+  </si>
+  <si>
+    <t>MAURITIUS</t>
+  </si>
+  <si>
+    <t>MEXICO</t>
+  </si>
+  <si>
+    <t>NETHERLANDS</t>
+  </si>
+  <si>
+    <t>NEW ZEALAND</t>
+  </si>
+  <si>
+    <t>NORWAY</t>
+  </si>
+  <si>
+    <t>PAKISTAN</t>
+  </si>
+  <si>
+    <t>PANAMA</t>
+  </si>
+  <si>
+    <t>PHILIPPINES</t>
+  </si>
+  <si>
+    <t>POLAND</t>
+  </si>
+  <si>
+    <t>PORTUGAL</t>
+  </si>
+  <si>
+    <t>RUSSIA</t>
+  </si>
+  <si>
+    <t>SAUDI ARABIA</t>
+  </si>
+  <si>
+    <t>SINGAPORE</t>
+  </si>
+  <si>
+    <t>SOUTH AFRICA</t>
+  </si>
+  <si>
+    <t>SOUTH KOREA</t>
+  </si>
+  <si>
+    <t>SPAIN</t>
+  </si>
+  <si>
+    <t>SRI LANKA</t>
+  </si>
+  <si>
+    <t>SWEDEN</t>
+  </si>
+  <si>
+    <t>SWITZERLAND</t>
+  </si>
+  <si>
+    <t>TAIWAN</t>
+  </si>
+  <si>
+    <t>THE NETHERLANDS</t>
+  </si>
+  <si>
+    <t>TURKEY</t>
+  </si>
+  <si>
+    <t>U.A.E</t>
+  </si>
+  <si>
+    <t>UNITED ARAB EMIRATES</t>
+  </si>
+  <si>
+    <t>UNITED KINGDOM</t>
+  </si>
+  <si>
+    <t>UNITED STATES</t>
+  </si>
+  <si>
+    <t>VIETNAM</t>
   </si>
 </sst>
 </file>
@@ -826,7 +952,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="MASTER_COUNTRY" displayName="MASTER_COUNTRY" ref="L1:L12" headerRowCount="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="MASTER_COUNTRY" displayName="MASTER_COUNTRY" ref="L1:L53" headerRowCount="0">
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="SHIPTO_COUNTRY"/>
   </tableColumns>
@@ -1169,7 +1295,7 @@
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A1" s="40" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="B1" s="40"/>
       <c r="C1" s="40"/>
@@ -10849,7 +10975,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr defaultRowHeight="13.8" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5" customWidth="1"/>
@@ -10883,7 +11009,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="C2" t="s">
         <v>36</v>
@@ -10901,330 +11027,497 @@
         <v>40</v>
       </c>
       <c r="L2" s="28" t="s">
-        <v>41</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="C3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" t="s">
         <v>42</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="G3" s="27" t="s">
+      <c r="H3" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="H3" s="27" t="s">
+      <c r="J3" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="J3" s="29" t="s">
-        <v>46</v>
-      </c>
       <c r="L3" s="28" t="s">
-        <v>47</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G4" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="E4" t="s">
+      <c r="H4" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="G4" s="27" t="s">
+      <c r="J4" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="H4" s="27" t="s">
-        <v>51</v>
-      </c>
-      <c r="J4" s="28" t="s">
-        <v>52</v>
-      </c>
       <c r="L4" s="29" t="s">
-        <v>53</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="C5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G5" s="27" t="s">
+        <v>53</v>
+      </c>
+      <c r="H5" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="E5" t="s">
+      <c r="J5" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="G5" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="H5" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="J5" s="29" t="s">
-        <v>58</v>
-      </c>
       <c r="L5" s="29" t="s">
-        <v>59</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="G6" s="27" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H6" s="27" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="J6" s="28" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="L6" s="28" t="s">
-        <v>63</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="G7" s="27" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="H7" s="27" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J7" s="29" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="L7" s="29" t="s">
-        <v>66</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="27"/>
       <c r="G8" s="27" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="H8" s="27" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="J8" s="28" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="L8" s="28" t="s">
-        <v>69</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="27"/>
       <c r="C9" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="G9" s="27" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="H9" s="27" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J9" s="29" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="L9" s="28" t="s">
-        <v>72</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="27"/>
       <c r="C10" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G10" s="27" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="H10" s="27" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="J10" s="28" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="L10" s="28" t="s">
-        <v>75</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="27"/>
       <c r="C11" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="G11" s="27" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="H11" s="27" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="J11" s="28" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="L11" s="29" t="s">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="G12" s="27" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="H12" s="27" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J12" s="28" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="L12" s="30" t="s">
-        <v>84</v>
+        <v>121</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="G13" s="27" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="H13" s="27" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J13" s="31" t="s">
-        <v>87</v>
+        <v>77</v>
+      </c>
+      <c r="L13" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="G14" s="27" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="H14" s="27" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J14" s="28" t="s">
-        <v>89</v>
+        <v>79</v>
+      </c>
+      <c r="L14" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="G15" s="27" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="H15" s="27" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="J15" s="29" t="s">
-        <v>92</v>
+        <v>82</v>
+      </c>
+      <c r="L15" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="G16" s="27" t="s">
+        <v>83</v>
+      </c>
+      <c r="H16" s="27" t="s">
+        <v>84</v>
+      </c>
+      <c r="J16" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="L16" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="17" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="G17" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="H17" s="27" t="s">
+        <v>87</v>
+      </c>
+      <c r="J17" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="L17" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="G18" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="H18" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="J18" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="L18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="19" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J19" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="L19" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="20" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J20" s="28" t="s">
+        <v>91</v>
+      </c>
+      <c r="L20" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="21" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J21" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="L21" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="22" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J22" s="28" t="s">
         <v>93</v>
       </c>
-      <c r="H16" s="27" t="s">
+      <c r="L22" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="23" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J23" s="28" t="s">
         <v>94</v>
       </c>
-      <c r="J16" s="28" t="s">
+      <c r="L23" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="24" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J24" s="28" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="17" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="G17" s="27" t="s">
+      <c r="L24" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="25" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J25" s="29" t="s">
         <v>96</v>
       </c>
-      <c r="H17" s="27" t="s">
+      <c r="L25" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="26" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J26" s="28" t="s">
         <v>97</v>
       </c>
-      <c r="J17" s="29" t="s">
+      <c r="L26" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="27" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J27" s="29" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="18" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="G18" s="27" t="s">
-        <v>71</v>
-      </c>
-      <c r="H18" s="27" t="s">
-        <v>45</v>
-      </c>
-      <c r="J18" s="28" t="s">
+      <c r="L27" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="28" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J28" s="28" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="19" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="J19" s="29" t="s">
+      <c r="L28" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="29" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J29" s="29" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="20" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="J20" s="28" t="s">
+      <c r="L29" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="30" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J30" s="29" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="21" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="J21" s="29" t="s">
+      <c r="L30" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="31" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="J31" s="32" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="22" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="J22" s="28" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="23" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="J23" s="28" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="24" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="J24" s="28" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="25" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="J25" s="29" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="26" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="J26" s="28" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="27" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="J27" s="29" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="28" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="J28" s="28" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="29" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="J29" s="29" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="30" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="J30" s="29" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="31" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="J31" s="32" t="s">
-        <v>112</v>
+      <c r="L31" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="32" spans="7:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L32" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="33" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L33" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="34" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L34" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="35" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L35" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="36" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L36" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="37" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L37" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="38" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L38" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="39" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L39" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="40" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L40" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="41" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L41" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="42" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L42" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="43" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L43" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="44" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L44" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="45" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L45" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="46" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L46" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="47" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L47" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="48" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L48" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="49" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L49" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="50" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L50" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="51" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L51" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="52" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L52" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="53" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L53" t="s">
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update download templates (data validation) for NYG / GW / EA
Replace all three BU templates with the updated data-validation versions.
The template-version hash changes with file content, so users who downloaded
an older copy will see the "template updated — please re-download" hint.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/air-request-template_EA.xlsx
+++ b/public/air-request-template_EA.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C06D01C9-4811-452F-8960-D616630FC553}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3380EBFC-201A-4A17-80F5-FE60DC130CBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="157">
   <si>
     <t>LOGISTICS</t>
   </si>
@@ -128,9 +128,6 @@
     <t>G</t>
   </si>
   <si>
-    <t>GMT_TYPE</t>
-  </si>
-  <si>
     <t>AIRPORT</t>
   </si>
   <si>
@@ -146,9 +143,6 @@
     <t>SHORTS</t>
   </si>
   <si>
-    <t>BOTTC</t>
-  </si>
-  <si>
     <t>Los Angeles</t>
   </si>
   <si>
@@ -158,12 +152,6 @@
     <t>EA</t>
   </si>
   <si>
-    <t>JACKET,Hoodie</t>
-  </si>
-  <si>
-    <t>JKT</t>
-  </si>
-  <si>
     <t>Chicago</t>
   </si>
   <si>
@@ -173,12 +161,6 @@
     <t>TRM</t>
   </si>
   <si>
-    <t>TANK,T-shirt</t>
-  </si>
-  <si>
-    <t>OVS</t>
-  </si>
-  <si>
     <t>Melbourne</t>
   </si>
   <si>
@@ -191,18 +173,12 @@
     <t>POLO SHIRT</t>
   </si>
   <si>
-    <t>POL</t>
-  </si>
-  <si>
     <t>Toronto</t>
   </si>
   <si>
     <t>BOXER</t>
   </si>
   <si>
-    <t>UNDER</t>
-  </si>
-  <si>
     <t>Vancouver</t>
   </si>
   <si>
@@ -215,9 +191,6 @@
     <t>Hong Kong</t>
   </si>
   <si>
-    <t xml:space="preserve">BOXER </t>
-  </si>
-  <si>
     <t>Amsterdam</t>
   </si>
   <si>
@@ -239,60 +212,39 @@
     <t>PANTS</t>
   </si>
   <si>
-    <t>BOTTB</t>
-  </si>
-  <si>
     <t>DURHAM</t>
   </si>
   <si>
     <t>PRODUCTION</t>
   </si>
   <si>
-    <t>JACKET,PULLOVER,SWEATSHIRT</t>
-  </si>
-  <si>
     <t>LOCKBOURN</t>
   </si>
   <si>
     <t>COMMERCIAL</t>
   </si>
   <si>
-    <t>PULLOVER,SWEATSHIRT</t>
-  </si>
-  <si>
     <t>SEATTLE WA, USA</t>
   </si>
   <si>
-    <t>JACKET,SWEATSHIRT,PULLOVER</t>
-  </si>
-  <si>
     <t>PEARSON INT,CANADA</t>
   </si>
   <si>
     <t>HEADBAND</t>
   </si>
   <si>
-    <t>ELAST</t>
-  </si>
-  <si>
     <t>MIAMI,USA</t>
   </si>
   <si>
     <t>GLOVES</t>
   </si>
   <si>
-    <t>GLO</t>
-  </si>
-  <si>
     <t>ATLANTA,USA</t>
   </si>
   <si>
     <t>SLEEVES</t>
   </si>
   <si>
-    <t>OTHER</t>
-  </si>
-  <si>
     <t>DALLAS,FORT WORTH INT,USA</t>
   </si>
   <si>
@@ -516,6 +468,36 @@
   </si>
   <si>
     <t>VIETNAM</t>
+  </si>
+  <si>
+    <t>DRIFIT SLEEVES</t>
+  </si>
+  <si>
+    <t>HEAD TIE</t>
+  </si>
+  <si>
+    <t>HOODIE</t>
+  </si>
+  <si>
+    <t>JACKET</t>
+  </si>
+  <si>
+    <t>KNITTED POLO SHIRT</t>
+  </si>
+  <si>
+    <t>KNITTED SHIRT</t>
+  </si>
+  <si>
+    <t>NECKWRAP</t>
+  </si>
+  <si>
+    <t>SLEEVE</t>
+  </si>
+  <si>
+    <t>SWEATSHIRT</t>
+  </si>
+  <si>
+    <t>TANK</t>
   </si>
 </sst>
 </file>
@@ -942,7 +924,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="MASTER_GARMENT_TYPE" displayName="MASTER_GARMENT_TYPE" ref="G1:H18" headerRowCount="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="MASTER_GARMENT_TYPE" displayName="MASTER_GARMENT_TYPE" ref="G1:H21" headerRowCount="0">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="DESCRIPTION"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="GMT_TYPE"/>
@@ -1295,7 +1277,7 @@
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A1" s="40" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="B1" s="40"/>
       <c r="C1" s="40"/>
@@ -10997,527 +10979,500 @@
       <c r="G1" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="24"/>
+      <c r="J1" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="J1" s="25" t="s">
+      <c r="L1" s="26" t="s">
         <v>34</v>
-      </c>
-      <c r="L1" s="26" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s">
         <v>36</v>
       </c>
-      <c r="E2" t="s">
-        <v>37</v>
-      </c>
       <c r="G2" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="H2" s="27"/>
+      <c r="J2" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="H2" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="J2" s="28" t="s">
-        <v>40</v>
-      </c>
       <c r="L2" s="28" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G3" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="H3" s="27"/>
+      <c r="J3" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="E3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G3" s="27" t="s">
-        <v>43</v>
-      </c>
-      <c r="H3" s="27" t="s">
-        <v>44</v>
-      </c>
-      <c r="J3" s="29" t="s">
-        <v>45</v>
-      </c>
       <c r="L3" s="28" t="s">
-        <v>112</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="C4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="E4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G4" s="27" t="s">
-        <v>48</v>
-      </c>
-      <c r="H4" s="27" t="s">
-        <v>49</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="H4" s="27"/>
       <c r="J4" s="28" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="L4" s="29" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="E5" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="G5" s="27" t="s">
-        <v>53</v>
-      </c>
-      <c r="H5" s="27" t="s">
-        <v>54</v>
-      </c>
+        <v>148</v>
+      </c>
+      <c r="H5" s="27"/>
       <c r="J5" s="29" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="L5" s="29" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="G6" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="H6" s="27" t="s">
-        <v>57</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="H6" s="27"/>
       <c r="J6" s="28" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="L6" s="28" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="G7" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="H7" s="27" t="s">
-        <v>49</v>
-      </c>
+        <v>149</v>
+      </c>
+      <c r="H7" s="27"/>
       <c r="J7" s="29" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="L7" s="29" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="27"/>
       <c r="G8" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="H8" s="27" t="s">
-        <v>57</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="H8" s="27"/>
       <c r="J8" s="28" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="L8" s="28" t="s">
-        <v>117</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="27"/>
       <c r="C9" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="G9" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="H9" s="27" t="s">
-        <v>49</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="H9" s="27"/>
       <c r="J9" s="29" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="L9" s="28" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="27"/>
       <c r="C10" t="s">
+        <v>87</v>
+      </c>
+      <c r="G10" s="27" t="s">
+        <v>152</v>
+      </c>
+      <c r="H10" s="27"/>
+      <c r="J10" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="L10" s="28" t="s">
         <v>103</v>
-      </c>
-      <c r="G10" s="27" t="s">
-        <v>66</v>
-      </c>
-      <c r="H10" s="27" t="s">
-        <v>66</v>
-      </c>
-      <c r="J10" s="28" t="s">
-        <v>67</v>
-      </c>
-      <c r="L10" s="28" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="27"/>
       <c r="C11" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="G11" s="27" t="s">
-        <v>69</v>
-      </c>
-      <c r="H11" s="27" t="s">
-        <v>70</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="H11" s="27"/>
       <c r="J11" s="28" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="L11" s="29" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="G12" s="27" t="s">
-        <v>73</v>
-      </c>
-      <c r="H12" s="27" t="s">
-        <v>44</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="H12" s="27"/>
       <c r="J12" s="28" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="L12" s="30" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="G13" s="27" t="s">
-        <v>76</v>
-      </c>
-      <c r="H13" s="27" t="s">
-        <v>49</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="H13" s="27"/>
       <c r="J13" s="31" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="L13" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="G14" s="27" t="s">
-        <v>78</v>
-      </c>
-      <c r="H14" s="27" t="s">
-        <v>44</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="H14" s="27"/>
       <c r="J14" s="28" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="L14" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="G15" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="H15" s="27" t="s">
-        <v>81</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="H15" s="27"/>
       <c r="J15" s="29" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="L15" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="G16" s="27" t="s">
-        <v>83</v>
-      </c>
-      <c r="H16" s="27" t="s">
-        <v>84</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="H16" s="27"/>
       <c r="J16" s="28" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="L16" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="17" spans="7:12" x14ac:dyDescent="0.25">
       <c r="G17" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="H17" s="27" t="s">
-        <v>87</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="H17" s="27"/>
       <c r="J17" s="29" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="L17" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18" spans="7:12" x14ac:dyDescent="0.25">
       <c r="G18" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="H18" s="27" t="s">
-        <v>44</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="H18" s="27"/>
       <c r="J18" s="28" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="L18" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
     </row>
     <row r="19" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="G19" t="s">
+        <v>155</v>
+      </c>
       <c r="J19" s="29" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="L19" t="s">
-        <v>128</v>
+        <v>112</v>
       </c>
     </row>
     <row r="20" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="G20" t="s">
+        <v>51</v>
+      </c>
       <c r="J20" s="28" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="L20" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
     </row>
     <row r="21" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="G21" t="s">
+        <v>156</v>
+      </c>
       <c r="J21" s="29" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="L21" t="s">
-        <v>130</v>
+        <v>114</v>
       </c>
     </row>
     <row r="22" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J22" s="28" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="L22" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
     </row>
     <row r="23" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J23" s="28" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="L23" t="s">
-        <v>132</v>
+        <v>116</v>
       </c>
     </row>
     <row r="24" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J24" s="28" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="L24" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
     </row>
     <row r="25" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J25" s="29" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="L25" t="s">
-        <v>134</v>
+        <v>118</v>
       </c>
     </row>
     <row r="26" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J26" s="28" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="L26" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
     </row>
     <row r="27" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J27" s="29" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="L27" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
     </row>
     <row r="28" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J28" s="28" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="L28" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
     </row>
     <row r="29" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J29" s="29" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="L29" t="s">
-        <v>138</v>
+        <v>122</v>
       </c>
     </row>
     <row r="30" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J30" s="29" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="L30" t="s">
-        <v>139</v>
+        <v>123</v>
       </c>
     </row>
     <row r="31" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J31" s="32" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="L31" t="s">
-        <v>140</v>
+        <v>124</v>
       </c>
     </row>
     <row r="32" spans="7:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L32" t="s">
-        <v>141</v>
+        <v>125</v>
       </c>
     </row>
     <row r="33" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L33" t="s">
-        <v>142</v>
+        <v>126</v>
       </c>
     </row>
     <row r="34" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L34" t="s">
-        <v>143</v>
+        <v>127</v>
       </c>
     </row>
     <row r="35" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L35" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
     </row>
     <row r="36" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L36" t="s">
-        <v>145</v>
+        <v>129</v>
       </c>
     </row>
     <row r="37" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L37" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
     </row>
     <row r="38" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L38" t="s">
-        <v>147</v>
+        <v>131</v>
       </c>
     </row>
     <row r="39" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L39" t="s">
-        <v>148</v>
+        <v>132</v>
       </c>
     </row>
     <row r="40" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L40" t="s">
-        <v>149</v>
+        <v>133</v>
       </c>
     </row>
     <row r="41" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L41" t="s">
-        <v>150</v>
+        <v>134</v>
       </c>
     </row>
     <row r="42" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L42" t="s">
-        <v>151</v>
+        <v>135</v>
       </c>
     </row>
     <row r="43" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L43" t="s">
-        <v>152</v>
+        <v>136</v>
       </c>
     </row>
     <row r="44" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L44" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
     </row>
     <row r="45" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L45" t="s">
-        <v>154</v>
+        <v>138</v>
       </c>
     </row>
     <row r="46" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L46" t="s">
-        <v>155</v>
+        <v>139</v>
       </c>
     </row>
     <row r="47" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L47" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
     </row>
     <row r="48" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L48" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
     </row>
     <row r="49" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L49" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
     </row>
     <row r="50" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L50" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
     </row>
     <row r="51" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L51" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
     </row>
     <row r="52" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L52" t="s">
-        <v>161</v>
+        <v>145</v>
       </c>
     </row>
     <row r="53" spans="12:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L53" t="s">
-        <v>162</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>